<commit_message>
cleanup: remove superseded sec_2_2_2_okishio.md (replaced by sec_2_2_3)
</commit_message>
<xml_diff>
--- a/data/raw/Chile/distr_19202024.xlsx
+++ b/data/raw/Chile/distr_19202024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ReposGitHub\Capacity-Utilization-US_Chile\data\raw\Chile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C29C412F-7705-411F-B082-245524579A1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DB49C95-2E88-4FD3-BB9E-B913F7E335CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{BB82A50C-484D-49A8-91E5-2427640CBBEB}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Periodo</t>
   </si>
@@ -62,6 +62,9 @@
   </si>
   <si>
     <t>psh</t>
+  </si>
+  <si>
+    <t>periodo</t>
   </si>
 </sst>
 </file>
@@ -3752,7 +3755,7 @@
         <v>0.51859563721870416</v>
       </c>
       <c r="D67" s="6">
-        <f t="shared" ref="D67:D107" si="3">C67/B67</f>
+        <f t="shared" ref="D67:D106" si="3">C67/B67</f>
         <v>1.0772557901688657</v>
       </c>
     </row>
@@ -4082,7 +4085,7 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
-        <f t="shared" ref="A87:A107" si="4">A86+1</f>
+        <f t="shared" ref="A87:A106" si="4">A86+1</f>
         <v>2005</v>
       </c>
       <c r="B87" s="4">
@@ -4460,7 +4463,7 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>5</v>

</xml_diff>